<commit_message>
:wqConsolidate codebase to root and prepare for cloud Docker deployment:wq :wq
</commit_message>
<xml_diff>
--- a/results/IBM_Interview_Results.xlsx
+++ b/results/IBM_Interview_Results.xlsx
@@ -533,7 +533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S5"/>
+  <dimension ref="A1:T11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -555,6 +555,7 @@
     <col width="19" customWidth="1" min="17" max="17"/>
     <col width="19" customWidth="1" min="18" max="18"/>
     <col width="27" customWidth="1" min="19" max="19"/>
+    <col width="20" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -965,6 +966,517 @@
       <c r="S5" s="13" t="inlineStr">
         <is>
           <t>Terminated – Tab Switch</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-07-17T10:42:57.523939</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>ravi.kumar@ibm.com</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1999-01-01</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Vivek Goyal</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>vigoyal5@in.ibm.com</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="N6" s="8" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q6" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="R6" s="8" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="S6" s="4" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-17T10:52:00.817592</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>ravi.kumar@ibm.com</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>1999-01-01</t>
+        </is>
+      </c>
+      <c r="F7" s="12" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="inlineStr">
+        <is>
+          <t>Vivek Goyal</t>
+        </is>
+      </c>
+      <c r="H7" s="12" t="inlineStr">
+        <is>
+          <t>vigoyal5@in.ibm.com</t>
+        </is>
+      </c>
+      <c r="I7" s="12" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="J7" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="K7" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="L7" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="M7" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="N7" s="8" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="O7" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="P7" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q7" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="R7" s="8" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="S7" s="13" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="T7" s="13" t="inlineStr">
+        <is>
+          <t>Recorded &amp; Saved</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-07-17T13:19:33.456550</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>ravi.kumar@ibm.com</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>1999-01-01</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Vivek Goyal</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>vigoyal5@in.ibm.com</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M8" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="N8" s="8" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q8" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="R8" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="S8" s="4" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="T8" s="4" t="inlineStr">
+        <is>
+          <t>Recorded &amp; Saved</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-17T13:27:11.756010</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>ravi.kumar@ibm.com</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>1999-01-01</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G9" s="12" t="inlineStr">
+        <is>
+          <t>Vivek Goyal</t>
+        </is>
+      </c>
+      <c r="H9" s="12" t="inlineStr">
+        <is>
+          <t>vigoyal5@in.ibm.com</t>
+        </is>
+      </c>
+      <c r="I9" s="12" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="J9" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="K9" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="L9" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="M9" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="N9" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="O9" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="P9" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q9" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="R9" s="8" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="S9" s="13" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="T9" s="13" t="inlineStr">
+        <is>
+          <t>Recorded &amp; Saved</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-07-17T13:35:25.289678</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>RAVI KUMAR</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ravi.kumar@ibm.com</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>1994-08-02</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>VIVEK GOYAL</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>vigoyal5@in.ibm.com</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M10" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="N10" s="8" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q10" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="R10" s="8" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="S10" s="4" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="T10" s="4" t="inlineStr">
+        <is>
+          <t>Recorded &amp; Saved</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-17T13:42:33.377468</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>ravi.kumar@ibm.com</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>1999-01-01</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G11" s="12" t="inlineStr">
+        <is>
+          <t>Vivek Goyal</t>
+        </is>
+      </c>
+      <c r="H11" s="12" t="inlineStr">
+        <is>
+          <t>vigoyal5@in.ibm.com</t>
+        </is>
+      </c>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="J11" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="K11" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="L11" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="M11" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="N11" s="8" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="O11" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="P11" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" s="8" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="S11" s="13" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="T11" s="13" t="inlineStr">
+        <is>
+          <t>Recorded &amp; Saved</t>
         </is>
       </c>
     </row>
@@ -979,7 +1491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I79"/>
+  <dimension ref="A1:I176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4292,6 +4804,4050 @@
         </is>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B80" s="10" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C80" s="10" t="inlineStr">
+        <is>
+          <t>--- Section A: Job Description Questions ---</t>
+        </is>
+      </c>
+      <c r="D80" s="10" t="inlineStr"/>
+      <c r="E80" s="10" t="inlineStr"/>
+      <c r="F80" s="10" t="inlineStr"/>
+      <c r="G80" s="10" t="inlineStr"/>
+      <c r="H80" s="10" t="inlineStr"/>
+      <c r="I80" s="10" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>5</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>1</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>In Selenium WebDriver with Java, which method is used to locate an element by its CSS selector?</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>driver.getElement(By.cssSelector("#elementId"))</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>driver.findElement(By.cssSelector("#elementId"))</t>
+        </is>
+      </c>
+      <c r="I81" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>5</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>2</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>You need to execute automated test scripts in a CI/CD pipeline using Jenkins. Which of the following is the correct approach to integrate your Maven-based Selenium project?</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Configure a Jenkins job with 'Invoke top-level Maven targets' and specify 'clean test' as the goal</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Configure a Jenkins job with 'Invoke top-level Maven targets' and specify 'clean test' as the goal</t>
+        </is>
+      </c>
+      <c r="I82" s="6" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>5</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>3</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Which TestNG annotation is used to execute a method before each test method in a test class?</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>@BeforeClass</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>@BeforeMethod</t>
+        </is>
+      </c>
+      <c r="I83" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>5</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C84" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>4</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>In a Page Object Model (POM) framework, you have the following code:
+```java
+public class LoginPage {
+    WebDriver driver;
+    By usernameField = By.id("username");
+    By passwordField = By.id("password");
+    By loginButton = By.xpath("//button[@type='submit']");
+    public void login(String user, String pass) {
+        driver.findElement(usernameField).sendKeys(user);
+        driver.findElement(passwordField).sendKeys(pass);
+        driver.findElement(loginButton).click();
+    }
+}
+```
+What is missing from this implementation?</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>The return statement in the login method</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>The constructor to initialize the WebDriver instance</t>
+        </is>
+      </c>
+      <c r="I84" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>5</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C85" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>5</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>When performing API automation testing using Rest Assured in Java, which method is used to validate the HTTP response status code?</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>given().when().get("/api/users").then().checkStatus(200)</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>given().when().get("/api/users").then().assertThat().statusCode(200)</t>
+        </is>
+      </c>
+      <c r="I85" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>5</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C86" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>6</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Your Selenium test suite is failing intermittently with 'StaleElementReferenceException'. The test navigates to a page, clicks a button that triggers a DOM update, and then tries to interact with an element. What is the most appropriate solution?</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Add Thread.sleep(5000) before interacting with the element</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Implement WebDriverWait with ExpectedConditions to wait for element to be clickable after DOM update</t>
+        </is>
+      </c>
+      <c r="I86" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>5</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C87" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>7</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>In Maven, which file contains the project dependencies and build configuration for a Java Selenium automation project?</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>dependencies.config</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>pom.xml</t>
+        </is>
+      </c>
+      <c r="I87" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>5</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C88" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>8</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>You are working in an Agile Scrum team and need to automate test cases for a new user story. During which Agile ceremony should you discuss the testability and automation approach for this story?</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Sprint Retrospective</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Sprint Planning and Refinement</t>
+        </is>
+      </c>
+      <c r="I88" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>5</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C89" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>9</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Which Git command is used to create a new branch and switch to it immediately for developing automation scripts?</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>git branch new-feature &amp;&amp; git checkout new-feature</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>git checkout -b new-feature</t>
+        </is>
+      </c>
+      <c r="I89" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>5</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C90" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>10</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Your automation suite needs to validate data in a MySQL database after a web transaction. You have a test scenario where a user registration should insert a record. Which approach is most appropriate?</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Manually check the database using MySQL Workbench after test execution</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Use JDBC to connect to database, execute SELECT query with user details, and validate the result set</t>
+        </is>
+      </c>
+      <c r="I90" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="B91" s="11" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C91" s="11" t="inlineStr">
+        <is>
+          <t>--- Section B: Resume Questions ---</t>
+        </is>
+      </c>
+      <c r="D91" s="11" t="inlineStr"/>
+      <c r="E91" s="11" t="inlineStr"/>
+      <c r="F91" s="11" t="inlineStr"/>
+      <c r="G91" s="11" t="inlineStr"/>
+      <c r="H91" s="11" t="inlineStr"/>
+      <c r="I91" s="11" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>5</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C92" s="7" t="inlineStr">
+        <is>
+          <t>Section B</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>11</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Your resume mentions you developed a Selenium automation framework using Page Object Model (POM). In POM, if you have a login page with username, password fields and a submit button, which of the following best describes how you would structure the LoginPage class to handle dynamic waits for the submit button that appears only after both fields are filled?</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Initialize WebElement submitButton with @FindBy and use WebDriverWait with ExpectedConditions.elementToBeClickable() in the clickSubmit() method</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Initialize WebElement submitButton with @FindBy and use WebDriverWait with ExpectedConditions.elementToBeClickable() in the clickSubmit() method</t>
+        </is>
+      </c>
+      <c r="I92" s="6" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>5</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C93" s="7" t="inlineStr">
+        <is>
+          <t>Section B</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>12</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Your resume states you automated over 1,000 regression test cases with TestNG. When running parallel execution in TestNG, you notice intermittent failures due to shared test data. Which TestNG configuration approach would best resolve this issue while maintaining parallel execution?</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Use parallel="tests" and create a singleton pattern for test data management</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Set parallel="methods" in testng.xml and use @BeforeMethod to initialize fresh test data for each method</t>
+        </is>
+      </c>
+      <c r="I93" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>5</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C94" s="7" t="inlineStr">
+        <is>
+          <t>Section B</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>13</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Your resume mentions you developed API automation scripts using Rest Assured. Given this Rest Assured code snippet:
+```java
+given()
+  .contentType(ContentType.JSON)
+  .body(requestBody)
+.when()
+  .post("/api/users")
+.then()
+  .statusCode(201)
+  .body("user.id", notNullValue())
+  .body("user.email", equalTo("test@example.com"));
+```
+What would be the most efficient way to extract and store the user.id value for use in subsequent API calls?</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Parse the entire response as String and use regex to extract the id</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Use .extract().path("user.id") after .then() and store in a variable</t>
+        </is>
+      </c>
+      <c r="I94" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>5</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C95" s="7" t="inlineStr">
+        <is>
+          <t>Section B</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>14</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Your resume highlights that you integrated the automation suite with Jenkins CI/CD pipeline and reduced regression testing from 5 days to 1 day. In a scenario where your Jenkins job randomly fails with 'StaleElementReferenceException' during nightly runs but passes when run manually, what is the most likely root cause and solution?</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Jenkins server has insufficient memory; increase heap size in Jenkins configuration</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>DOM is being refreshed during test execution; implement retry logic with WebDriverWait or relocate elements</t>
+        </is>
+      </c>
+      <c r="I95" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>5</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C96" s="7" t="inlineStr">
+        <is>
+          <t>Section B</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>15</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Your resume mentions you worked closely with Developers, Product Owners, and Business Analysts in an Agile environment and reduced production defects by 30%. During a sprint, a critical bug is found in production on Friday evening. The fix requires a hotfix deployment, but your automation suite takes 8 hours to run. As the Senior Test Automation Engineer, what would be your recommended approach?</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Ask developers to write unit tests for the fix and skip automation testing for hotfixes</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Identify and execute only smoke tests and tests related to the affected module, then deploy with monitoring</t>
+        </is>
+      </c>
+      <c r="I96" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="B97" s="10" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C97" s="10" t="inlineStr">
+        <is>
+          <t>--- Section A: Job Description Questions ---</t>
+        </is>
+      </c>
+      <c r="D97" s="10" t="inlineStr"/>
+      <c r="E97" s="10" t="inlineStr"/>
+      <c r="F97" s="10" t="inlineStr"/>
+      <c r="G97" s="10" t="inlineStr"/>
+      <c r="H97" s="10" t="inlineStr"/>
+      <c r="I97" s="10" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>6</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C98" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>1</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>In Selenium WebDriver with Java, which method is used to locate an element by its CSS selector?</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>driver.findElement(By.css("#elementId"))</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>driver.findElement(By.cssSelector("#elementId"))</t>
+        </is>
+      </c>
+      <c r="I98" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>6</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C99" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>2</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Which TestNG annotation is used to execute a method before each test method in a test class?</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>@BeforeMethod</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>@BeforeMethod</t>
+        </is>
+      </c>
+      <c r="I99" s="6" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>6</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C100" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>3</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>You need to automate a test that verifies API response status code is 200. Which Rest Assured code snippet correctly implements this?
+```java
+Response response = given()
+    .when()
+    .get("/api/users");
+```</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>response.assertStatusCode(200);</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>response.then().assertThat().statusCode(200);</t>
+        </is>
+      </c>
+      <c r="I100" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>6</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>4</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>In a Page Object Model (POM) framework, what is the primary purpose of using the @FindBy annotation in Selenium with Java?</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>To declare and locate web elements on a page</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>To declare and locate web elements on a page</t>
+        </is>
+      </c>
+      <c r="I101" s="6" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>6</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C102" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>5</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>You are creating a data-driven test framework. Which Maven dependency configuration correctly adds TestNG and Apache POI for reading Excel test data?
+```xml
+&lt;dependencies&gt;
+    &lt;!-- Option content here --&gt;
+&lt;/dependencies&gt;
+```</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>&lt;dependency&gt;&lt;groupId&gt;testng&lt;/groupId&gt;&lt;artifactId&gt;testng-framework&lt;/artifactId&gt;&lt;/dependency&gt;
+&lt;dependency&gt;&lt;groupId&gt;apache.poi&lt;/groupId&gt;&lt;artifactId&gt;excel-reader&lt;/artifactId&gt;&lt;/dependency&gt;</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>&lt;dependency&gt;&lt;groupId&gt;org.testng&lt;/groupId&gt;&lt;artifactId&gt;testng&lt;/artifactId&gt;&lt;/dependency&gt;
+&lt;dependency&gt;&lt;groupId&gt;org.apache.poi&lt;/groupId&gt;&lt;artifactId&gt;poi-ooxml&lt;/artifactId&gt;&lt;/dependency&gt;</t>
+        </is>
+      </c>
+      <c r="I102" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>6</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C103" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>6</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Your Selenium test fails intermittently with 'StaleElementReferenceException'. What is the most likely cause and solution?</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Element is not visible; use explicit wait with ExpectedConditions.visibilityOfElementLocated()</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>DOM has been refreshed after element was located; re-locate the element before interacting</t>
+        </is>
+      </c>
+      <c r="I103" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>6</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C104" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>7</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>In a CI/CD pipeline using Jenkins, you need to trigger automated Selenium tests after every code commit. Which Jenkins feature should you configure?</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Post-build Actions with 'Archive artifacts'</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Build Triggers with 'Poll SCM' or 'GitHub webhook'</t>
+        </is>
+      </c>
+      <c r="I104" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>6</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C105" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>8</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Your team is implementing Agile methodology. During which Agile ceremony should you, as a Test Automation Engineer, present automation test results and discuss testing blockers?</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Sprint Planning</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Daily Stand-up</t>
+        </is>
+      </c>
+      <c r="I105" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>6</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C106" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>9</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>You need to validate database records after a web application transaction. Which Java code snippet correctly executes a SQL query using JDBC?
+```java
+Connection conn = DriverManager.getConnection(url, user, password);
+```</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>ResultSet rs = conn.executeQuery("SELECT * FROM users");</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Statement stmt = conn.createStatement();
+ResultSet rs = stmt.executeQuery("SELECT * FROM users");</t>
+        </is>
+      </c>
+      <c r="I106" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>6</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>10</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>A junior team member asks for your guidance on choosing between TestNG and JUnit for a new automation project. As a senior engineer, what is the most important factor you should consider?</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>The choice doesn't matter as both frameworks are identical</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Project requirements, team expertise, and existing framework compatibility</t>
+        </is>
+      </c>
+      <c r="I107" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="B108" s="11" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C108" s="11" t="inlineStr">
+        <is>
+          <t>--- Section B: Resume Questions ---</t>
+        </is>
+      </c>
+      <c r="D108" s="11" t="inlineStr"/>
+      <c r="E108" s="11" t="inlineStr"/>
+      <c r="F108" s="11" t="inlineStr"/>
+      <c r="G108" s="11" t="inlineStr"/>
+      <c r="H108" s="11" t="inlineStr"/>
+      <c r="I108" s="11" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>6</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C109" s="7" t="inlineStr">
+        <is>
+          <t>Section B</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>11</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Your resume mentions you developed a Selenium automation framework using Java, TestNG, and Maven. In TestNG, you need to execute a specific test method only when another test method passes. Which annotation combination would you use?</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>@Test(dependsOnMethods = "testMethodName")</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>@Test(dependsOnMethods = "testMethodName")</t>
+        </is>
+      </c>
+      <c r="I109" s="6" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>6</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C110" s="7" t="inlineStr">
+        <is>
+          <t>Section B</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>12</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Your resume states you automated over 1,000 regression test cases and implemented parallel execution using TestNG. Given this TestNG XML configuration snippet:
+```xml
+&lt;suite name="Suite" parallel="methods" thread-count="5"&gt;
+  &lt;test name="Test"&gt;
+    &lt;classes&gt;
+      &lt;class name="TestClass"/&gt;
+    &lt;/classes&gt;
+  &lt;/test&gt;
+&lt;/suite&gt;
+```
+What will be the execution behavior?</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Only @BeforeMethod and @AfterMethod will run in parallel</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>All test methods within TestClass will run in parallel with maximum 5 threads</t>
+        </is>
+      </c>
+      <c r="I110" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>6</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C111" s="7" t="inlineStr">
+        <is>
+          <t>Section B</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>13</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Your resume mentions you developed API automation scripts using Rest Assured. You need to validate that a POST request to create a user returns status 201 and the response body contains a specific user ID. Which Rest Assured code is correct?</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>when().post("/users").then().statusCode(201).extract().response().body("id");</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>given().body(user).when().post("/users").then().statusCode(201).body("id", equalTo(123));</t>
+        </is>
+      </c>
+      <c r="I111" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>6</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C112" s="7" t="inlineStr">
+        <is>
+          <t>Section B</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>14</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Your resume highlights that you designed a Page Object Model (POM) framework. In your Digital Banking Platform project, you have a login page with dynamic elements that load after AJAX calls. Which Selenium WebDriver approach would you implement in your POM class to handle this scenario most effectively?</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>Set implicit wait to 30 seconds globally in the base page class</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>Implement WebDriverWait with ExpectedConditions.visibilityOfElementLocated() for dynamic elements</t>
+        </is>
+      </c>
+      <c r="I112" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>6</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C113" s="7" t="inlineStr">
+        <is>
+          <t>Section B</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>15</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Your resume states you worked closely with Developers, Product Owners, and Business Analysts in an Agile environment and reduced regression testing effort from 5 days to 1 day. During a sprint, developers delivered a critical feature on the last day, but your automation suite detected 15 high-priority defects. The Product Owner wants to release anyway. How would you handle this situation?</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>Immediately escalate to senior management and refuse to sign off on the release until all defects are fixed</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>Present defect severity data, risk analysis, and potential business impact to stakeholders; facilitate a collaborative decision on release vs. fix priority</t>
+        </is>
+      </c>
+      <c r="I113" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="B114" s="10" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C114" s="10" t="inlineStr">
+        <is>
+          <t>--- Section A: Job Description Questions ---</t>
+        </is>
+      </c>
+      <c r="D114" s="10" t="inlineStr"/>
+      <c r="E114" s="10" t="inlineStr"/>
+      <c r="F114" s="10" t="inlineStr"/>
+      <c r="G114" s="10" t="inlineStr"/>
+      <c r="H114" s="10" t="inlineStr"/>
+      <c r="I114" s="10" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>7</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C115" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>1</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>In Selenium WebDriver with Java, which method is used to switch the driver's focus to a specific frame using its index?</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>driver.selectFrame(int index)</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>driver.switchTo().frame(int index)</t>
+        </is>
+      </c>
+      <c r="I115" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>7</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C116" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>2</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>You need to create a Page Object Model (POM) class for a login page. Which annotation is used in Selenium to initialize web elements using PageFactory?</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>@Locator</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>@FindBy</t>
+        </is>
+      </c>
+      <c r="I116" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>7</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C117" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>3</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>In TestNG, which annotation should be used to execute a method once before all test methods in a test class?</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>@BeforeMethod</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>@BeforeTest</t>
+        </is>
+      </c>
+      <c r="I117" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>7</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C118" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>4</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>You are writing an API automation test using Rest Assured. Which method chain correctly sends a GET request and validates the status code is 200?
+```java
+RestAssured.baseURI = "https://api.example.com";
+// Complete the code
+```</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>given().when().get("/users").then().statusCode(200);</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>given().when().get("/users").then().statusCode(200);</t>
+        </is>
+      </c>
+      <c r="I118" s="6" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>7</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C119" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>5</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>In Maven, which file is used to define project dependencies, plugins, and build configurations?</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>config.properties</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>pom.xml</t>
+        </is>
+      </c>
+      <c r="I119" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>7</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C120" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>6</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Your Selenium test fails with 'StaleElementReferenceException'. What is the most likely cause of this exception?</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>The WebDriver session has expired</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>The element was located but is no longer attached to the DOM</t>
+        </is>
+      </c>
+      <c r="I120" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>7</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C121" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>7</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>You need to execute your Selenium test suite as part of a CI/CD pipeline. Which Jenkins plugin is commonly used to trigger Maven-based test execution?</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>Selenium Plugin</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>Maven Integration Plugin</t>
+        </is>
+      </c>
+      <c r="I121" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>7</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C122" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>8</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Your team is following Agile methodology. During which ceremony would you typically discuss and estimate the effort required for automating new test scenarios?</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Sprint Retrospective</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Sprint Planning</t>
+        </is>
+      </c>
+      <c r="I122" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>7</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C123" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>9</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>You are implementing a Data-Driven framework using TestNG. Which TestNG annotation is used to provide multiple sets of test data to a test method?</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>@DataProvider</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>@DataProvider</t>
+        </is>
+      </c>
+      <c r="I123" s="6" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>7</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C124" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>10</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>A critical production bug was found that your automated regression suite did not catch. As a Senior Test Automation Engineer, what is your FIRST responsibility?</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>Analyze why the existing test suite missed the bug and identify gaps in test coverage</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>Analyze why the existing test suite missed the bug and identify gaps in test coverage</t>
+        </is>
+      </c>
+      <c r="I124" s="6" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="B125" s="11" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C125" s="11" t="inlineStr">
+        <is>
+          <t>--- Section B: Resume Questions ---</t>
+        </is>
+      </c>
+      <c r="D125" s="11" t="inlineStr"/>
+      <c r="E125" s="11" t="inlineStr"/>
+      <c r="F125" s="11" t="inlineStr"/>
+      <c r="G125" s="11" t="inlineStr"/>
+      <c r="H125" s="11" t="inlineStr"/>
+      <c r="I125" s="11" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>7</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C126" s="7" t="inlineStr">
+        <is>
+          <t>Section B</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>11</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Your resume mentions you developed a Selenium automation framework using TestNG and Maven. In TestNG, if you want to execute test methods in a specific order within a test class, which annotation attribute should you use?</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="I126" s="6" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>7</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C127" s="7" t="inlineStr">
+        <is>
+          <t>Section B</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>12</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Your resume states you implemented Page Object Model (POM) framework. Given this Page Object class snippet:
+```java
+public class LoginPage {
+    WebDriver driver;
+    @FindBy(id="username")
+    WebElement usernameField;
+    public LoginPage(WebDriver driver) {
+        this.driver = driver;
+        // What is missing here?
+    }
+}
+```
+What critical line is missing in the constructor to make @FindBy annotations work?</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>new WebDriverWait(driver, 10);</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>PageFactory.initElements(driver, this);</t>
+        </is>
+      </c>
+      <c r="I127" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>7</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C128" s="7" t="inlineStr">
+        <is>
+          <t>Section B</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>13</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Your resume mentions you developed API automation scripts using Rest Assured. Which Rest Assured method chain correctly validates that a GET request to '/api/users/123' returns status code 200 and response time is less than 2000ms?</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>RestAssured.get("/api/users/123").then().status(200).responseTime(lessThan(2000));</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>given().when().get("/api/users/123").then().assertThat().statusCode(200).and().time(lessThan(2000L), MILLISECONDS);</t>
+        </is>
+      </c>
+      <c r="I128" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>7</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C129" s="7" t="inlineStr">
+        <is>
+          <t>Section B</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>14</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Your resume states you integrated automation suite with Jenkins CI/CD pipeline and implemented parallel execution using TestNG. In a scenario where 5 test classes need to run in parallel on Jenkins, but you notice tests are failing due to WebDriver instance conflicts, what is the most appropriate TestNG configuration to resolve this?</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>Set parallel="methods" and thread-count="5" in testng.xml, use ThreadLocal&lt;WebDriver&gt; for driver instances</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>Set parallel="methods" and thread-count="5" in testng.xml, use ThreadLocal&lt;WebDriver&gt; for driver instances</t>
+        </is>
+      </c>
+      <c r="I129" s="6" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>7</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C130" s="7" t="inlineStr">
+        <is>
+          <t>Section B</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>15</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Your resume mentions you worked closely with Developers, Product Owners, and Business Analysts in an Agile environment and reduced regression testing effort from 5 days to 1 day. During a sprint, the Product Owner requests adding 15 new test scenarios, but the Development team is behind schedule and may not deliver features until the last day of the sprint. How should you prioritize your automation work?</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>Collaborate with PO to prioritize critical scenarios, automate high-priority ones incrementally as features are delivered, and defer low-priority ones to next sprint</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>Collaborate with PO to prioritize critical scenarios, automate high-priority ones incrementally as features are delivered, and defer low-priority ones to next sprint</t>
+        </is>
+      </c>
+      <c r="I130" s="6" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B131" s="10" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C131" s="10" t="inlineStr">
+        <is>
+          <t>--- Section A: Job Description Questions ---</t>
+        </is>
+      </c>
+      <c r="D131" s="10" t="inlineStr"/>
+      <c r="E131" s="10" t="inlineStr"/>
+      <c r="F131" s="10" t="inlineStr"/>
+      <c r="G131" s="10" t="inlineStr"/>
+      <c r="H131" s="10" t="inlineStr"/>
+      <c r="I131" s="10" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>8</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C132" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>1</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>In Selenium WebDriver with Java, which method is used to switch the driver's focus to a specific frame using its index?</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>driver.switchTo().frame(int index)</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>driver.switchTo().frame(int index)</t>
+        </is>
+      </c>
+      <c r="I132" s="6" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="n">
+        <v>8</v>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C133" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>2</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>You need to create a Page Object Model (POM) class for a login page. Which annotation should you use with PageFactory to initialize web elements in Selenium?</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>@FindElement</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>@FindBy</t>
+        </is>
+      </c>
+      <c r="I133" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>8</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C134" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>3</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Which TestNG annotation is used to execute a method before each test method in a test class?</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>@BeforeClass</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>@BeforeMethod</t>
+        </is>
+      </c>
+      <c r="I134" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>8</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C135" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>4</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>You are automating API tests using Rest Assured in Java. Which method chain correctly sends a GET request and validates the status code is 200?
+```java
+RestAssured.baseURI = "https://api.example.com";
+// Complete the code
+```</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>given().when().get("/users").then().statusCode(200);</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>given().when().get("/users").then().statusCode(200);</t>
+        </is>
+      </c>
+      <c r="I135" s="6" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>8</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C136" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>5</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Your automation suite is integrated with Jenkins CI/CD pipeline. After a test execution, 5 out of 50 tests failed. The Product Owner asks you to prioritize which failures to investigate first. What should be your approach?</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>Check if failures are in critical user journeys, verify if they are consistent across runs, and review recent code changes</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>Check if failures are in critical user journeys, verify if they are consistent across runs, and review recent code changes</t>
+        </is>
+      </c>
+      <c r="I136" s="6" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="B137" s="11" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C137" s="11" t="inlineStr">
+        <is>
+          <t>--- Section B: Resume Questions ---</t>
+        </is>
+      </c>
+      <c r="D137" s="11" t="inlineStr"/>
+      <c r="E137" s="11" t="inlineStr"/>
+      <c r="F137" s="11" t="inlineStr"/>
+      <c r="G137" s="11" t="inlineStr"/>
+      <c r="H137" s="11" t="inlineStr"/>
+      <c r="I137" s="11" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>8</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C138" s="7" t="inlineStr">
+        <is>
+          <t>Section B</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>6</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Your resume mentions you developed a Selenium automation framework using TestNG and Maven. In TestNG, which annotation would you use to execute a method before each test method in a test class?</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>@BeforeSuite</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>@BeforeMethod</t>
+        </is>
+      </c>
+      <c r="I138" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>8</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C139" s="7" t="inlineStr">
+        <is>
+          <t>Section B</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>7</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Your resume states you implemented Page Object Model (POM) framework. Given this code snippet:
+```java
+public class LoginPage {
+    WebDriver driver;
+    @FindBy(id="username")
+    WebElement usernameField;
+    public LoginPage(WebDriver driver) {
+        this.driver = driver;
+        // What is missing here?
+    }
+}
+```
+What is the missing critical step to make @FindBy annotations work?</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>PageFactory.initElements(driver, this);</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>PageFactory.initElements(driver, this);</t>
+        </is>
+      </c>
+      <c r="I139" s="6" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="n">
+        <v>8</v>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C140" s="7" t="inlineStr">
+        <is>
+          <t>Section B</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>8</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Your resume mentions you developed API automation scripts using Rest Assured. Which Rest Assured method chain correctly validates that a GET request to '/users/123' returns status code 200 and contains a field 'name' with value 'John'?</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>when().get("/users/123").expect().statusCode(200).body("name", is("John"));</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>given().when().get("/users/123").then().statusCode(200).body("name", equalTo("John"));</t>
+        </is>
+      </c>
+      <c r="I140" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>8</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C141" s="7" t="inlineStr">
+        <is>
+          <t>Section B</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>9</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Your resume states you integrated automation suite with Jenkins CI/CD pipeline and implemented parallel execution using TestNG. In a scenario where 5 test classes need to run in parallel on Jenkins with 3 available nodes, and each test takes 10 minutes sequentially, what is the minimum total execution time if parallel execution is optimally configured?</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>50 minutes</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>20 minutes</t>
+        </is>
+      </c>
+      <c r="I141" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>8</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C142" s="7" t="inlineStr">
+        <is>
+          <t>Section B</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>10</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Your resume mentions you worked closely with Developers, Product Owners, and Business Analysts in an Agile environment and reduced regression testing effort from 5 days to 1 day. What was likely the MOST critical factor in achieving this 80% reduction?</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>Reducing the scope of regression testing by removing low-priority test cases</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>Implementing comprehensive automation coverage with parallel execution and CI/CD integration</t>
+        </is>
+      </c>
+      <c r="I142" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B143" s="10" t="inlineStr">
+        <is>
+          <t>RAVI KUMAR</t>
+        </is>
+      </c>
+      <c r="C143" s="10" t="inlineStr">
+        <is>
+          <t>--- Section A: Job Description Questions ---</t>
+        </is>
+      </c>
+      <c r="D143" s="10" t="inlineStr"/>
+      <c r="E143" s="10" t="inlineStr"/>
+      <c r="F143" s="10" t="inlineStr"/>
+      <c r="G143" s="10" t="inlineStr"/>
+      <c r="H143" s="10" t="inlineStr"/>
+      <c r="I143" s="10" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>9</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>RAVI KUMAR</t>
+        </is>
+      </c>
+      <c r="C144" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>1</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>In Selenium WebDriver with Java, which method is used to switch the driver's focus to a specific frame using its index?</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>driver.selectFrame(int index)</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>driver.switchTo().frame(int index)</t>
+        </is>
+      </c>
+      <c r="I144" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>9</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>RAVI KUMAR</t>
+        </is>
+      </c>
+      <c r="C145" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>2</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Which TestNG annotation is used to execute a method before each test method in a test class?</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>@BeforeMethod</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>@BeforeMethod</t>
+        </is>
+      </c>
+      <c r="I145" s="6" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>9</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>RAVI KUMAR</t>
+        </is>
+      </c>
+      <c r="C146" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>3</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>In a Page Object Model (POM) framework, you have a login page class. Which approach correctly implements the page factory pattern?
+```java
+public class LoginPage {
+    WebDriver driver;
+    // Option A
+    @FindBy(id = "username")
+    WebElement usernameField;
+    public LoginPage(WebDriver driver) {
+        this.driver = driver;
+        PageFactory.initElements(driver, this);
+    }
+}
+```</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>PageFactory.initElements should be called before assigning driver</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>The code is correct and follows Page Factory pattern properly</t>
+        </is>
+      </c>
+      <c r="I146" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>9</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>RAVI KUMAR</t>
+        </is>
+      </c>
+      <c r="C147" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>4</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>You need to perform API testing using Rest Assured. Which code snippet correctly sends a GET request and validates the status code is 200?
+```java
+// Option A
+RestAssured.given()
+    .when().get("/api/users")
+    .then().statusCode(200);
+```</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>Should use .post() instead of .get() for validation</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>The code is correct</t>
+        </is>
+      </c>
+      <c r="I147" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>9</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>RAVI KUMAR</t>
+        </is>
+      </c>
+      <c r="C148" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>5</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>In Maven, which file is used to define project dependencies, plugins, and build configurations?</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>config.properties</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>pom.xml</t>
+        </is>
+      </c>
+      <c r="I148" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>9</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>RAVI KUMAR</t>
+        </is>
+      </c>
+      <c r="C149" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>6</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Your Selenium test fails intermittently with 'StaleElementReferenceException'. The element exists but the test fails randomly. What is the most likely cause and solution?</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>WebDriver session has expired; restart the browser</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>Page is refreshing or DOM is being updated; implement explicit wait or re-locate element</t>
+        </is>
+      </c>
+      <c r="I149" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>9</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>RAVI KUMAR</t>
+        </is>
+      </c>
+      <c r="C150" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>7</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>You are integrating your Selenium automation suite with Jenkins CI/CD pipeline. Which Jenkins plugin is specifically designed for executing Maven-based test projects?</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>Git Plugin</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>Maven Integration Plugin</t>
+        </is>
+      </c>
+      <c r="I150" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>9</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>RAVI KUMAR</t>
+        </is>
+      </c>
+      <c r="C151" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>8</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Your team is following Agile Scrum methodology. During Sprint Planning, the Product Owner presents a new user story requiring automation. As a Senior Test Automation Engineer, what should be your immediate responsibility?</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>Analyze requirements, ask clarifying questions, estimate effort, and identify testable scenarios</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>Analyze requirements, ask clarifying questions, estimate effort, and identify testable scenarios</t>
+        </is>
+      </c>
+      <c r="I151" s="6" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>9</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>RAVI KUMAR</t>
+        </is>
+      </c>
+      <c r="C152" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>9</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>You need to validate data in a MySQL database after executing a test. Which Java code snippet correctly establishes a database connection and executes a SELECT query?
+```java
+// Option A
+Connection conn = DriverManager.getConnection(url, user, password);
+Statement stmt = conn.createStatement();
+ResultSet rs = stmt.executeQuery("SELECT * FROM users WHERE id=1");
+```</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>Should use PreparedStatement instead of Statement for all queries</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>The code is correct</t>
+        </is>
+      </c>
+      <c r="I152" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>9</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>RAVI KUMAR</t>
+        </is>
+      </c>
+      <c r="C153" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>10</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Your automation framework uses a Data-Driven approach with TestNG. You have test data in an Excel file. Which TestNG feature allows you to parameterize tests and run them with multiple data sets?</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>@DataProvider annotation with a method returning Object[][]</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>@DataProvider annotation with a method returning Object[][]</t>
+        </is>
+      </c>
+      <c r="I153" s="6" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B154" s="11" t="inlineStr">
+        <is>
+          <t>RAVI KUMAR</t>
+        </is>
+      </c>
+      <c r="C154" s="11" t="inlineStr">
+        <is>
+          <t>--- Section B: Resume Questions ---</t>
+        </is>
+      </c>
+      <c r="D154" s="11" t="inlineStr"/>
+      <c r="E154" s="11" t="inlineStr"/>
+      <c r="F154" s="11" t="inlineStr"/>
+      <c r="G154" s="11" t="inlineStr"/>
+      <c r="H154" s="11" t="inlineStr"/>
+      <c r="I154" s="11" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>9</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>RAVI KUMAR</t>
+        </is>
+      </c>
+      <c r="C155" s="7" t="inlineStr">
+        <is>
+          <t>Section B</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>11</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Your resume mentions you developed a Selenium automation framework using Java, TestNG, and Maven. In TestNG, which annotation would you use to execute a method before each test method in a test class?</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>@BeforeTest</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>@BeforeMethod</t>
+        </is>
+      </c>
+      <c r="I155" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>9</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>RAVI KUMAR</t>
+        </is>
+      </c>
+      <c r="C156" s="7" t="inlineStr">
+        <is>
+          <t>Section B</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>12</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Your resume states you automated over 1,000 regression test cases with 85% automation coverage. When implementing Page Object Model in Selenium, which approach correctly initializes web elements?
+```java
+public class LoginPage {
+    WebDriver driver;
+    // Which initialization is correct?
+}
+```</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>@FindBy(id = "user") WebElement username; with PageFactory.initElements()</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>@FindBy(id = "user") WebElement username; with PageFactory.initElements()</t>
+        </is>
+      </c>
+      <c r="I156" s="6" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>9</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>RAVI KUMAR</t>
+        </is>
+      </c>
+      <c r="C157" s="7" t="inlineStr">
+        <is>
+          <t>Section B</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>13</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Your resume mentions you developed API automation scripts using Rest Assured. Which Rest Assured code correctly validates that a GET response returns status 200 and contains a specific JSON field 'userId'?</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>given().get("/api/user").validate().status(200).field("userId").exists();</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>given().when().get("/api/user").then().statusCode(200).body("userId", notNullValue());</t>
+        </is>
+      </c>
+      <c r="I157" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="n">
+        <v>9</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>RAVI KUMAR</t>
+        </is>
+      </c>
+      <c r="C158" s="7" t="inlineStr">
+        <is>
+          <t>Section B</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>14</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Your resume states you integrated automation suite with Jenkins CI/CD pipeline and implemented parallel execution using TestNG. In a scenario where 5 test classes need to run in parallel on Jenkins with 3 available nodes, which TestNG configuration ensures optimal parallel execution?
+```xml
+&lt;suite name="RegressionSuite" parallel="?" thread-count="?"&gt;
+```</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>parallel="instances" thread-count="3"</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>parallel="classes" thread-count="3"</t>
+        </is>
+      </c>
+      <c r="I158" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>9</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>RAVI KUMAR</t>
+        </is>
+      </c>
+      <c r="C159" s="7" t="inlineStr">
+        <is>
+          <t>Section B</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>15</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Your resume mentions you worked closely with Developers, Product Owners, and Business Analysts in an Agile environment, reducing regression testing effort from 5 days to 1 day. During a sprint, a critical production bug is found 2 days before release. The Product Owner wants to add a new feature, but the Developer suggests fixing the bug first. As the Senior Test Automation Engineer, what would be your recommended approach?</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>Run both in parallel by splitting the team to meet all commitments</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>Support fixing the critical bug first, then assess if the feature can fit in the sprint</t>
+        </is>
+      </c>
+      <c r="I159" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="B160" s="10" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C160" s="10" t="inlineStr">
+        <is>
+          <t>--- Section A: Job Description Questions ---</t>
+        </is>
+      </c>
+      <c r="D160" s="10" t="inlineStr"/>
+      <c r="E160" s="10" t="inlineStr"/>
+      <c r="F160" s="10" t="inlineStr"/>
+      <c r="G160" s="10" t="inlineStr"/>
+      <c r="H160" s="10" t="inlineStr"/>
+      <c r="I160" s="10" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" t="n">
+        <v>10</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C161" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>1</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>In Selenium WebDriver with Java, which method is used to switch the driver's focus to a specific frame using its index?</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>driver.selectFrame(int index)</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>driver.switchTo().frame(int index)</t>
+        </is>
+      </c>
+      <c r="I161" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="n">
+        <v>10</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C162" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>2</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>You are designing a Page Object Model (POM) framework. Which annotation in TestNG would you use to execute a method before each test method in a test class?</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>@BeforeClass</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>@BeforeMethod</t>
+        </is>
+      </c>
+      <c r="I162" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="n">
+        <v>10</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C163" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>3</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>In Maven, which file contains project dependencies and build configuration?</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>settings.xml</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>pom.xml</t>
+        </is>
+      </c>
+      <c r="I163" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="n">
+        <v>10</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C164" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>4</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>Which Rest Assured method is used to send a GET request to an API endpoint and validate the response status code is 200?
+```java
+given().
+    baseUri("https://api.example.com").
+when().
+    get("/users").
+then().
+    ______;
+```</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>checkStatusCode(200)</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>statusCode(200)</t>
+        </is>
+      </c>
+      <c r="I164" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="n">
+        <v>10</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C165" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>5</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>Your automation suite needs to run tests on Chrome, Firefox, and Edge browsers. Which design pattern would you implement to initialize different browser drivers efficiently?</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>Observer Pattern</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>Factory Pattern</t>
+        </is>
+      </c>
+      <c r="I165" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="n">
+        <v>10</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C166" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>6</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>In a Data-Driven framework, you are reading test data from an Excel file. Which Java library is commonly used to read Excel files in Selenium automation?</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>Apache POI</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>Apache POI</t>
+        </is>
+      </c>
+      <c r="I166" s="6" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="n">
+        <v>10</v>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C167" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>7</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>You need to integrate your Selenium test suite with Jenkins for CI/CD. Which Jenkins plugin is specifically designed to execute Maven projects?</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>TestNG Plugin</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>Maven Integration Plugin</t>
+        </is>
+      </c>
+      <c r="I167" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="n">
+        <v>10</v>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C168" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>8</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>Your test script fails with 'StaleElementReferenceException' after the page dynamically updates. What is the most appropriate solution?</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>Use Thread.sleep() before clicking the element</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>Re-locate the element after the page update before interacting with it</t>
+        </is>
+      </c>
+      <c r="I168" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="n">
+        <v>10</v>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C169" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>9</v>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>During a sprint, the Product Owner requests adding 15 new test scenarios, but only 3 days remain. As a Senior Test Automation Engineer, what is your best approach?</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>Prioritize scenarios based on business impact and risk, automate critical ones first, and discuss capacity with the team</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>Prioritize scenarios based on business impact and risk, automate critical ones first, and discuss capacity with the team</t>
+        </is>
+      </c>
+      <c r="I169" s="6" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="n">
+        <v>10</v>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C170" s="5" t="inlineStr">
+        <is>
+          <t>Section A</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>10</v>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>In Git, which command would you use to create a new branch named 'feature-automation' and switch to it immediately?</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>git checkout -b feature-automation</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>git checkout -b feature-automation</t>
+        </is>
+      </c>
+      <c r="I170" s="6" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B171" s="11" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C171" s="11" t="inlineStr">
+        <is>
+          <t>--- Section B: Resume Questions ---</t>
+        </is>
+      </c>
+      <c r="D171" s="11" t="inlineStr"/>
+      <c r="E171" s="11" t="inlineStr"/>
+      <c r="F171" s="11" t="inlineStr"/>
+      <c r="G171" s="11" t="inlineStr"/>
+      <c r="H171" s="11" t="inlineStr"/>
+      <c r="I171" s="11" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" t="n">
+        <v>10</v>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C172" s="7" t="inlineStr">
+        <is>
+          <t>Section B</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>11</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Your resume mentions you developed a Selenium automation framework using Java, TestNG, and Maven. In TestNG, which annotation would you use to execute a method once before all test methods in a test class?</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>@BeforeTest</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>@BeforeClass</t>
+        </is>
+      </c>
+      <c r="I172" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="n">
+        <v>10</v>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C173" s="7" t="inlineStr">
+        <is>
+          <t>Section B</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>12</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>Your resume states you implemented Page Object Model (POM) framework. Given this LoginPage class snippet:
+```java
+public class LoginPage {
+    WebDriver driver;
+    @FindBy(id="username")
+    WebElement usernameField;
+    public LoginPage(WebDriver driver) {
+        this.driver = driver;
+        // What is missing here?
+    }
+}
+```
+What is the missing critical step in the constructor?</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>driver.manage().timeouts().implicitlyWait(10, TimeUnit.SECONDS)</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>PageFactory.initElements(driver, this)</t>
+        </is>
+      </c>
+      <c r="I173" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="n">
+        <v>10</v>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C174" s="7" t="inlineStr">
+        <is>
+          <t>Section B</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>13</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>Your resume mentions you developed API automation scripts using Rest Assured. Which Rest Assured method chain correctly validates that a GET request to '/users/123' returns status code 200 and contains a field 'name' with value 'John'?</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>given().get("/users/123").expect().statusCode(200).body("name", is("John"))</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>given().when().get("/users/123").then().statusCode(200).body("name", equalTo("John"))</t>
+        </is>
+      </c>
+      <c r="I174" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="n">
+        <v>10</v>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C175" s="7" t="inlineStr">
+        <is>
+          <t>Section B</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>14</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>Your resume states you integrated automation suite with Jenkins CI/CD pipeline and implemented parallel execution using TestNG. In a scenario where 5 test classes need to run in parallel on Jenkins with 3 available nodes, and each test takes 10 minutes sequentially, what is the minimum execution time achievable with optimal parallel configuration?</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>10 minutes</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>20 minutes</t>
+        </is>
+      </c>
+      <c r="I175" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="n">
+        <v>10</v>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Ravi Kumar</t>
+        </is>
+      </c>
+      <c r="C176" s="7" t="inlineStr">
+        <is>
+          <t>Section B</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>15</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>Your resume mentions you worked closely with Developers, Product Owners, and Business Analysts in an Agile environment and reduced regression testing effort from 5 days to 1 day. During a sprint, a critical production bug is found 2 days before release. The Product Owner wants to add a new feature, but the Developer suggests fixing the bug first. As the Senior Test Automation Engineer, what should be your recommended approach?</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>Recommend releasing as planned and fixing the bug in a hotfix after release</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>Support fixing the critical bug first, assess regression impact, and defer the feature to next sprint</t>
+        </is>
+      </c>
+      <c r="I176" s="8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>